<commit_message>
Manuscript branch snapshot: validation suite, appendices, and .zenodo.json
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/manuscript/validation_counts 2.xlsx
+++ b/manuscript/validation_counts 2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/scBiomarkers/bernd/cytometry/CyFj11/manuscript/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/System/Volumes/Data/pasteur/helix/projects/scBiomarkers/bernd/cytometry/CyFj11/manuscript/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF486D7A-EC04-8049-AA12-E819F9B122D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8900D7E-310A-1B42-8E12-492F214DDEAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1760" yWindow="600" windowWidth="38400" windowHeight="19320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51200" yWindow="0" windowWidth="19080" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1 - validation_counts" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="191">
   <si>
     <t>validation_counts</t>
   </si>
@@ -631,12 +631,36 @@
   <si>
     <t>Fj11 remake</t>
   </si>
+  <si>
+    <t>FJ11 cannot read even the file saved by FJ10, misinterpretes the ellipse gate and crashes</t>
+  </si>
+  <si>
+    <t>counts are correct, but the axis is not biexp but linear</t>
+  </si>
+  <si>
+    <t>counts are correct, but the axis is not log but linear</t>
+  </si>
+  <si>
+    <t>counts are correct, but the axis is not asinh but linear</t>
+  </si>
+  <si>
+    <t>ArcTanh, but no parameters</t>
+  </si>
+  <si>
+    <t>ellipse gate not correctly imported</t>
+  </si>
+  <si>
+    <t>not gate is only on PE_hi</t>
+  </si>
+  <si>
+    <t>we get 2 not gates for FITC_hi and PE_hi</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -664,6 +688,22 @@
     <font>
       <sz val="10"/>
       <color indexed="8"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <name val="Helvetica Neue"/>
       <family val="2"/>
     </font>
@@ -908,16 +948,16 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="11"/>
+        <color rgb="FFA5A5A5"/>
       </left>
       <right style="thin">
-        <color indexed="10"/>
+        <color rgb="FFA5A5A5"/>
       </right>
       <top style="thin">
-        <color indexed="11"/>
+        <color rgb="FFA5A5A5"/>
       </top>
       <bottom style="thin">
-        <color indexed="10"/>
+        <color rgb="FFA5A5A5"/>
       </bottom>
       <diagonal/>
     </border>
@@ -927,7 +967,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -997,16 +1037,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -2142,8 +2194,8 @@
   <dimension ref="A1:M105"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.33203125" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="105.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="19" style="1" customWidth="1"/>
+    <col min="1" max="1" width="6.83203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="11.33203125" style="1" customWidth="1"/>
     <col min="3" max="3" width="13.1640625" style="1" customWidth="1"/>
     <col min="4" max="4" width="8.83203125" style="1" customWidth="1"/>
     <col min="5" max="5" width="20.6640625" style="1" customWidth="1"/>
@@ -2571,7 +2623,7 @@
       <c r="H24" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="I24" s="24" t="s">
+      <c r="I24" s="23" t="s">
         <v>182</v>
       </c>
       <c r="J24" s="14" t="s">
@@ -2719,7 +2771,7 @@
         <v>4776</v>
       </c>
       <c r="H30" s="16">
-        <v>4778</v>
+        <v>4776</v>
       </c>
       <c r="I30" s="16">
         <v>4776</v>
@@ -2733,7 +2785,7 @@
       </c>
       <c r="L30" s="16" cm="1">
         <f t="array" ref="L30">F30-H30</f>
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="M30" s="12"/>
     </row>
@@ -2794,7 +2846,7 @@
         <v>4631</v>
       </c>
       <c r="H33" s="16">
-        <v>4636</v>
+        <v>4631</v>
       </c>
       <c r="I33" s="16">
         <v>4631</v>
@@ -2808,7 +2860,7 @@
       </c>
       <c r="L33" s="16" cm="1">
         <f t="array" ref="L33">F33-H33</f>
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="M33" s="12"/>
     </row>
@@ -2928,7 +2980,7 @@
       <c r="B39" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="C39" s="14" t="s">
+      <c r="C39" s="23" t="s">
         <v>61</v>
       </c>
       <c r="D39" s="14" t="s">
@@ -2941,24 +2993,24 @@
         <v>7301</v>
       </c>
       <c r="G39" s="16">
-        <v>7314</v>
+        <v>7306</v>
       </c>
       <c r="H39" s="16">
-        <v>7503</v>
+        <v>0</v>
       </c>
       <c r="I39" s="16">
         <v>7290</v>
       </c>
       <c r="J39" s="16">
-        <v>7217</v>
+        <v>7281</v>
       </c>
       <c r="K39" s="16" cm="1">
         <f t="array" ref="K39">F39-G39</f>
-        <v>-13</v>
+        <v>-5</v>
       </c>
       <c r="L39" s="16" cm="1">
         <f t="array" ref="L39">F39-H39</f>
-        <v>-202</v>
+        <v>7301</v>
       </c>
       <c r="M39" s="12"/>
     </row>
@@ -2972,7 +3024,9 @@
       <c r="E40" s="11"/>
       <c r="F40" s="11"/>
       <c r="G40" s="11"/>
-      <c r="H40" s="11"/>
+      <c r="H40" s="26" t="s">
+        <v>183</v>
+      </c>
       <c r="I40" s="11"/>
       <c r="J40" s="11"/>
       <c r="K40" s="11"/>
@@ -3022,10 +3076,10 @@
         <v>2403</v>
       </c>
       <c r="I42" s="16">
-        <v>2396</v>
-      </c>
-      <c r="J42" s="16">
-        <v>2396</v>
+        <v>2400</v>
+      </c>
+      <c r="J42" s="28">
+        <v>2400</v>
       </c>
       <c r="K42" s="16" cm="1">
         <f t="array" ref="K42">F42-G42</f>
@@ -3047,7 +3101,9 @@
       <c r="E43" s="11"/>
       <c r="F43" s="11"/>
       <c r="G43" s="11"/>
-      <c r="H43" s="11"/>
+      <c r="H43" s="26" t="s">
+        <v>184</v>
+      </c>
       <c r="I43" s="11"/>
       <c r="J43" s="11"/>
       <c r="K43" s="11"/>
@@ -3116,7 +3172,7 @@
       <c r="I46" s="16">
         <v>3198</v>
       </c>
-      <c r="J46" s="16">
+      <c r="J46" s="28">
         <v>3198</v>
       </c>
       <c r="K46" s="16" cm="1">
@@ -3139,7 +3195,9 @@
       <c r="E47" s="11"/>
       <c r="F47" s="11"/>
       <c r="G47" s="11"/>
-      <c r="H47" s="11"/>
+      <c r="H47" s="26" t="s">
+        <v>185</v>
+      </c>
       <c r="I47" s="11"/>
       <c r="J47" s="11"/>
       <c r="K47" s="11"/>
@@ -3191,7 +3249,7 @@
       <c r="I49" s="16">
         <v>1599</v>
       </c>
-      <c r="J49" s="16">
+      <c r="J49" s="28">
         <v>1599</v>
       </c>
       <c r="K49" s="16" cm="1">
@@ -3214,8 +3272,12 @@
       <c r="E50" s="11"/>
       <c r="F50" s="11"/>
       <c r="G50" s="11"/>
-      <c r="H50" s="11"/>
-      <c r="I50" s="11"/>
+      <c r="H50" s="26" t="s">
+        <v>186</v>
+      </c>
+      <c r="I50" s="26" t="s">
+        <v>187</v>
+      </c>
       <c r="J50" s="11"/>
       <c r="K50" s="11"/>
       <c r="L50" s="11"/>
@@ -3261,7 +3323,7 @@
         <v>9441</v>
       </c>
       <c r="H52" s="16">
-        <v>9462</v>
+        <v>9441</v>
       </c>
       <c r="I52" s="16">
         <v>9441</v>
@@ -3275,7 +3337,7 @@
       </c>
       <c r="L52" s="16" cm="1">
         <f t="array" ref="L52">F52-H52</f>
-        <v>-21</v>
+        <v>0</v>
       </c>
       <c r="M52" s="12"/>
     </row>
@@ -3302,7 +3364,7 @@
         <v>8800</v>
       </c>
       <c r="H53" s="16">
-        <v>8813</v>
+        <v>8800</v>
       </c>
       <c r="I53" s="16">
         <v>8800</v>
@@ -3316,7 +3378,7 @@
       </c>
       <c r="L53" s="16" cm="1">
         <f t="array" ref="L53">F53-H53</f>
-        <v>-13</v>
+        <v>0</v>
       </c>
       <c r="M53" s="12"/>
     </row>
@@ -3392,7 +3454,7 @@
         <v>7554</v>
       </c>
       <c r="H57" s="16">
-        <v>7562</v>
+        <v>7554</v>
       </c>
       <c r="I57" s="16">
         <v>7558</v>
@@ -3406,7 +3468,7 @@
       </c>
       <c r="L57" s="16" cm="1">
         <f t="array" ref="L57">F57-H57</f>
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="M57" s="12"/>
     </row>
@@ -3433,7 +3495,7 @@
         <v>7392</v>
       </c>
       <c r="H58" s="16">
-        <v>7419</v>
+        <v>7392</v>
       </c>
       <c r="I58" s="16">
         <v>7392</v>
@@ -3447,7 +3509,7 @@
       </c>
       <c r="L58" s="16" cm="1">
         <f t="array" ref="L58">F58-H58</f>
-        <v>-27</v>
+        <v>0</v>
       </c>
       <c r="M58" s="12"/>
     </row>
@@ -3474,7 +3536,7 @@
         <v>6979</v>
       </c>
       <c r="H59" s="16">
-        <v>7013</v>
+        <v>6979</v>
       </c>
       <c r="I59" s="16">
         <v>6983</v>
@@ -3488,7 +3550,7 @@
       </c>
       <c r="L59" s="16" cm="1">
         <f t="array" ref="L59">F59-H59</f>
-        <v>-34</v>
+        <v>0</v>
       </c>
       <c r="M59" s="12"/>
     </row>
@@ -3515,7 +3577,7 @@
         <v>7967</v>
       </c>
       <c r="H60" s="16">
-        <v>7968</v>
+        <v>7967</v>
       </c>
       <c r="I60" s="16">
         <v>7967</v>
@@ -3529,7 +3591,7 @@
       </c>
       <c r="L60" s="16" cm="1">
         <f t="array" ref="L60">F60-H60</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="M60" s="12"/>
     </row>
@@ -3556,7 +3618,7 @@
         <v>1021</v>
       </c>
       <c r="H61" s="16">
-        <v>987</v>
+        <v>1021</v>
       </c>
       <c r="I61" s="16">
         <v>1017</v>
@@ -3570,7 +3632,7 @@
       </c>
       <c r="L61" s="16" cm="1">
         <f t="array" ref="L61">F61-H61</f>
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="M61" s="12"/>
     </row>
@@ -3629,7 +3691,7 @@
         <v>9696</v>
       </c>
       <c r="H64" s="16">
-        <v>9705</v>
+        <v>9696</v>
       </c>
       <c r="I64" s="16">
         <v>9696</v>
@@ -3643,7 +3705,7 @@
       </c>
       <c r="L64" s="16" cm="1">
         <f t="array" ref="L64">F64-H64</f>
-        <v>-9</v>
+        <v>0</v>
       </c>
       <c r="M64" s="12"/>
     </row>
@@ -3670,7 +3732,7 @@
         <v>2897</v>
       </c>
       <c r="H65" s="16">
-        <v>2900</v>
+        <v>2897</v>
       </c>
       <c r="I65" s="16">
         <v>2897</v>
@@ -3684,7 +3746,7 @@
       </c>
       <c r="L65" s="16" cm="1">
         <f t="array" ref="L65">F65-H65</f>
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="M65" s="12"/>
     </row>
@@ -3711,7 +3773,7 @@
         <v>1930</v>
       </c>
       <c r="H66" s="16">
-        <v>1932</v>
+        <v>1930</v>
       </c>
       <c r="I66" s="16">
         <v>1930</v>
@@ -3725,7 +3787,7 @@
       </c>
       <c r="L66" s="16" cm="1">
         <f t="array" ref="L66">F66-H66</f>
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="M66" s="12"/>
     </row>
@@ -3926,7 +3988,7 @@
         <v>9765</v>
       </c>
       <c r="H73" s="16">
-        <v>9766</v>
+        <v>9765</v>
       </c>
       <c r="I73" s="16">
         <v>9765</v>
@@ -3940,7 +4002,7 @@
       </c>
       <c r="L73" s="16" cm="1">
         <f t="array" ref="L73">F73-H73</f>
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="M73" s="12"/>
     </row>
@@ -3967,13 +4029,13 @@
         <v>9797</v>
       </c>
       <c r="H74" s="16">
-        <v>9890</v>
+        <v>0</v>
       </c>
       <c r="I74" s="16">
         <v>9768</v>
       </c>
       <c r="J74" s="16">
-        <v>9759</v>
+        <v>9772</v>
       </c>
       <c r="K74" s="16" cm="1">
         <f t="array" ref="K74">F74-G74</f>
@@ -3981,7 +4043,7 @@
       </c>
       <c r="L74" s="16" cm="1">
         <f t="array" ref="L74">F74-H74</f>
-        <v>-87</v>
+        <v>9803</v>
       </c>
       <c r="M74" s="12"/>
     </row>
@@ -4030,7 +4092,7 @@
       <c r="A76" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="B76" s="26" t="s">
+      <c r="B76" s="24" t="s">
         <v>119</v>
       </c>
       <c r="C76" s="14" t="s">
@@ -4177,7 +4239,7 @@
       <c r="I79" s="16">
         <v>5934</v>
       </c>
-      <c r="J79" s="14" t="s">
+      <c r="J79" s="29" t="s">
         <v>130</v>
       </c>
       <c r="K79" s="16" cm="1">
@@ -4200,9 +4262,15 @@
       <c r="E80" s="11"/>
       <c r="F80" s="11"/>
       <c r="G80" s="11"/>
-      <c r="H80" s="11"/>
-      <c r="I80" s="11"/>
-      <c r="J80" s="11"/>
+      <c r="H80" s="27" t="s">
+        <v>188</v>
+      </c>
+      <c r="I80" s="26" t="s">
+        <v>189</v>
+      </c>
+      <c r="J80" s="26" t="s">
+        <v>190</v>
+      </c>
       <c r="K80" s="11"/>
       <c r="L80" s="11"/>
       <c r="M80" s="12"/>
@@ -4288,7 +4356,7 @@
         <v>9470</v>
       </c>
       <c r="H83" s="16">
-        <v>9486</v>
+        <v>9470</v>
       </c>
       <c r="I83" s="14" t="s">
         <v>137</v>
@@ -4302,7 +4370,7 @@
       </c>
       <c r="L83" s="16" cm="1">
         <f t="array" ref="L83">F83-H83</f>
-        <v>-16</v>
+        <v>0</v>
       </c>
       <c r="M83" s="12"/>
     </row>
@@ -4329,7 +4397,7 @@
         <v>2992</v>
       </c>
       <c r="H84" s="16">
-        <v>2158</v>
+        <v>0</v>
       </c>
       <c r="I84" s="14" t="s">
         <v>137</v>
@@ -4343,7 +4411,7 @@
       </c>
       <c r="L84" s="16" cm="1">
         <f t="array" ref="L84">F84-H84</f>
-        <v>825</v>
+        <v>2983</v>
       </c>
       <c r="M84" s="12"/>
     </row>
@@ -4370,7 +4438,7 @@
         <v>2838</v>
       </c>
       <c r="H85" s="16">
-        <v>2842</v>
+        <v>2838</v>
       </c>
       <c r="I85" s="14" t="s">
         <v>137</v>
@@ -4384,7 +4452,7 @@
       </c>
       <c r="L85" s="16" cm="1">
         <f t="array" ref="L85">F85-H85</f>
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="M85" s="12"/>
     </row>
@@ -4411,7 +4479,7 @@
         <v>1888</v>
       </c>
       <c r="H86" s="16">
-        <v>1891</v>
+        <v>1888</v>
       </c>
       <c r="I86" s="14" t="s">
         <v>137</v>
@@ -4425,7 +4493,7 @@
       </c>
       <c r="L86" s="16" cm="1">
         <f t="array" ref="L86">F86-H86</f>
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="M86" s="12"/>
     </row>
@@ -4578,10 +4646,10 @@
       <c r="H91" s="16">
         <v>19132</v>
       </c>
-      <c r="I91" s="16">
+      <c r="I91" s="28">
         <v>19132</v>
       </c>
-      <c r="J91" s="16">
+      <c r="J91" s="28">
         <v>19079</v>
       </c>
       <c r="K91" s="16" cm="1">
@@ -4592,7 +4660,10 @@
         <f t="array" ref="L91">F91-H91</f>
         <v>80</v>
       </c>
-      <c r="M91" s="12"/>
+      <c r="M91" s="12">
+        <f>I91-J91</f>
+        <v>53</v>
+      </c>
     </row>
     <row r="92" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A92" s="9" t="s">
@@ -4617,10 +4688,10 @@
       <c r="H92" s="16">
         <v>18594</v>
       </c>
-      <c r="I92" s="16">
+      <c r="I92" s="28">
         <v>18594</v>
       </c>
-      <c r="J92" s="16">
+      <c r="J92" s="28">
         <v>18545</v>
       </c>
       <c r="K92" s="16" cm="1">
@@ -4631,13 +4702,16 @@
         <f t="array" ref="L92">F92-H92</f>
         <v>95</v>
       </c>
-      <c r="M92" s="12"/>
+      <c r="M92" s="12">
+        <f t="shared" ref="M92:M105" si="0">I92-J92</f>
+        <v>49</v>
+      </c>
     </row>
     <row r="93" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A93" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="B93" s="26" t="s">
+      <c r="B93" s="24" t="s">
         <v>158</v>
       </c>
       <c r="C93" s="11"/>
@@ -4656,10 +4730,10 @@
       <c r="H93" s="16">
         <v>18466</v>
       </c>
-      <c r="I93" s="16">
+      <c r="I93" s="28">
         <v>18466</v>
       </c>
-      <c r="J93" s="16">
+      <c r="J93" s="28">
         <v>18418</v>
       </c>
       <c r="K93" s="16" cm="1">
@@ -4670,7 +4744,10 @@
         <f t="array" ref="L93">F93-H93</f>
         <v>107</v>
       </c>
-      <c r="M93" s="12"/>
+      <c r="M93" s="12">
+        <f t="shared" si="0"/>
+        <v>48</v>
+      </c>
     </row>
     <row r="94" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A94" s="9" t="s">
@@ -4695,11 +4772,11 @@
       <c r="H94" s="14" t="s">
         <v>163</v>
       </c>
-      <c r="I94" s="16">
-        <v>918</v>
-      </c>
-      <c r="J94" s="16">
-        <v>940</v>
+      <c r="I94" s="28">
+        <v>920</v>
+      </c>
+      <c r="J94" s="28">
+        <v>942</v>
       </c>
       <c r="K94" s="16" cm="1">
         <f t="array" ref="K94">F94-G94</f>
@@ -4709,7 +4786,10 @@
         <f t="array" ref="L94">F94-H94</f>
         <v>#VALUE!</v>
       </c>
-      <c r="M94" s="12"/>
+      <c r="M94" s="12">
+        <f t="shared" si="0"/>
+        <v>-22</v>
+      </c>
     </row>
     <row r="95" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A95" s="17"/>
@@ -4732,10 +4812,10 @@
       <c r="H95" s="14" t="s">
         <v>166</v>
       </c>
-      <c r="I95" s="16">
-        <v>310</v>
-      </c>
-      <c r="J95" s="16">
+      <c r="I95" s="28">
+        <v>312</v>
+      </c>
+      <c r="J95" s="28">
         <v>314</v>
       </c>
       <c r="K95" s="16" cm="1">
@@ -4746,7 +4826,10 @@
         <f t="array" ref="L95">F95-H95</f>
         <v>#VALUE!</v>
       </c>
-      <c r="M95" s="12"/>
+      <c r="M95" s="12">
+        <f t="shared" si="0"/>
+        <v>-2</v>
+      </c>
     </row>
     <row r="96" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A96" s="9" t="s">
@@ -4771,11 +4854,11 @@
       <c r="H96" s="14" t="s">
         <v>166</v>
       </c>
-      <c r="I96" s="16">
-        <v>536</v>
-      </c>
-      <c r="J96" s="16">
-        <v>552</v>
+      <c r="I96" s="28">
+        <v>533</v>
+      </c>
+      <c r="J96" s="28">
+        <v>545</v>
       </c>
       <c r="K96" s="16" cm="1">
         <f t="array" ref="K96">F96-G96</f>
@@ -4785,7 +4868,10 @@
         <f t="array" ref="L96">F96-H96</f>
         <v>#VALUE!</v>
       </c>
-      <c r="M96" s="12"/>
+      <c r="M96" s="12">
+        <f t="shared" si="0"/>
+        <v>-12</v>
+      </c>
     </row>
     <row r="97" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A97" s="17"/>
@@ -4808,11 +4894,11 @@
       <c r="H97" s="14" t="s">
         <v>166</v>
       </c>
-      <c r="I97" s="16">
-        <v>17448</v>
-      </c>
-      <c r="J97" s="16">
-        <v>17358</v>
+      <c r="I97" s="28">
+        <v>17357</v>
+      </c>
+      <c r="J97" s="28">
+        <v>17192</v>
       </c>
       <c r="K97" s="16" cm="1">
         <f t="array" ref="K97">F97-G97</f>
@@ -4822,7 +4908,10 @@
         <f t="array" ref="L97">F97-H97</f>
         <v>#VALUE!</v>
       </c>
-      <c r="M97" s="12"/>
+      <c r="M97" s="12">
+        <f t="shared" si="0"/>
+        <v>165</v>
+      </c>
     </row>
     <row r="98" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A98" s="17"/>
@@ -4845,11 +4934,11 @@
       <c r="H98" s="14" t="s">
         <v>166</v>
       </c>
-      <c r="I98" s="16">
-        <v>2461</v>
-      </c>
-      <c r="J98" s="16">
+      <c r="I98" s="28">
         <v>2452</v>
+      </c>
+      <c r="J98" s="28">
+        <v>2436</v>
       </c>
       <c r="K98" s="16" cm="1">
         <f t="array" ref="K98">F98-G98</f>
@@ -4859,7 +4948,10 @@
         <f t="array" ref="L98">F98-H98</f>
         <v>#VALUE!</v>
       </c>
-      <c r="M98" s="12"/>
+      <c r="M98" s="12">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
     </row>
     <row r="99" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A99" s="17"/>
@@ -4882,11 +4974,11 @@
       <c r="H99" s="14" t="s">
         <v>166</v>
       </c>
-      <c r="I99" s="16">
+      <c r="I99" s="28">
         <v>10746</v>
       </c>
-      <c r="J99" s="16">
-        <v>10747</v>
+      <c r="J99" s="28">
+        <v>10672</v>
       </c>
       <c r="K99" s="16" cm="1">
         <f t="array" ref="K99">F99-G99</f>
@@ -4896,7 +4988,10 @@
         <f t="array" ref="L99">F99-H99</f>
         <v>#VALUE!</v>
       </c>
-      <c r="M99" s="12"/>
+      <c r="M99" s="12">
+        <f t="shared" si="0"/>
+        <v>74</v>
+      </c>
     </row>
     <row r="100" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A100" s="17"/>
@@ -4919,11 +5014,11 @@
       <c r="H100" s="14" t="s">
         <v>166</v>
       </c>
-      <c r="I100" s="16">
-        <v>9195</v>
-      </c>
-      <c r="J100" s="16">
-        <v>9182</v>
+      <c r="I100" s="28">
+        <v>9165</v>
+      </c>
+      <c r="J100" s="28">
+        <v>9113</v>
       </c>
       <c r="K100" s="16" cm="1">
         <f t="array" ref="K100">F100-G100</f>
@@ -4933,7 +5028,10 @@
         <f t="array" ref="L100">F100-H100</f>
         <v>#VALUE!</v>
       </c>
-      <c r="M100" s="12"/>
+      <c r="M100" s="12">
+        <f t="shared" si="0"/>
+        <v>52</v>
+      </c>
     </row>
     <row r="101" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A101" s="17"/>
@@ -4956,11 +5054,11 @@
       <c r="H101" s="14" t="s">
         <v>166</v>
       </c>
-      <c r="I101" s="16">
-        <v>7482</v>
-      </c>
-      <c r="J101" s="16">
-        <v>7469</v>
+      <c r="I101" s="28">
+        <v>7462</v>
+      </c>
+      <c r="J101" s="28">
+        <v>7411</v>
       </c>
       <c r="K101" s="16" cm="1">
         <f t="array" ref="K101">F101-G101</f>
@@ -4970,7 +5068,10 @@
         <f t="array" ref="L101">F101-H101</f>
         <v>#VALUE!</v>
       </c>
-      <c r="M101" s="12"/>
+      <c r="M101" s="12">
+        <f t="shared" si="0"/>
+        <v>51</v>
+      </c>
     </row>
     <row r="102" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A102" s="17"/>
@@ -4993,11 +5094,11 @@
       <c r="H102" s="14" t="s">
         <v>166</v>
       </c>
-      <c r="I102" s="16">
-        <v>1412</v>
-      </c>
-      <c r="J102" s="16">
-        <v>1413</v>
+      <c r="I102" s="28">
+        <v>1407</v>
+      </c>
+      <c r="J102" s="28">
+        <v>1403</v>
       </c>
       <c r="K102" s="16" cm="1">
         <f t="array" ref="K102">F102-G102</f>
@@ -5007,7 +5108,10 @@
         <f t="array" ref="L102">F102-H102</f>
         <v>#VALUE!</v>
       </c>
-      <c r="M102" s="12"/>
+      <c r="M102" s="12">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
     </row>
     <row r="103" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A103" s="17"/>
@@ -5030,11 +5134,11 @@
       <c r="H103" s="14" t="s">
         <v>166</v>
       </c>
-      <c r="I103" s="16">
-        <v>265</v>
-      </c>
-      <c r="J103" s="16">
-        <v>264</v>
+      <c r="I103" s="28">
+        <v>261</v>
+      </c>
+      <c r="J103" s="28">
+        <v>263</v>
       </c>
       <c r="K103" s="16" cm="1">
         <f t="array" ref="K103">F103-G103</f>
@@ -5044,7 +5148,10 @@
         <f t="array" ref="L103">F103-H103</f>
         <v>#VALUE!</v>
       </c>
-      <c r="M103" s="12"/>
+      <c r="M103" s="12">
+        <f t="shared" si="0"/>
+        <v>-2</v>
+      </c>
     </row>
     <row r="104" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A104" s="17"/>
@@ -5067,10 +5174,10 @@
       <c r="H104" s="14" t="s">
         <v>166</v>
       </c>
-      <c r="I104" s="16">
+      <c r="I104" s="28">
         <v>6</v>
       </c>
-      <c r="J104" s="16">
+      <c r="J104" s="28">
         <v>7</v>
       </c>
       <c r="K104" s="16" cm="1">
@@ -5081,7 +5188,10 @@
         <f t="array" ref="L104">F104-H104</f>
         <v>#VALUE!</v>
       </c>
-      <c r="M104" s="12"/>
+      <c r="M104" s="12">
+        <f t="shared" si="0"/>
+        <v>-1</v>
+      </c>
     </row>
     <row r="105" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A105" s="18"/>
@@ -5104,11 +5214,11 @@
       <c r="H105" s="21" t="s">
         <v>166</v>
       </c>
-      <c r="I105" s="22">
-        <v>1470</v>
-      </c>
-      <c r="J105" s="22">
-        <v>1470</v>
+      <c r="I105" s="30">
+        <v>1466</v>
+      </c>
+      <c r="J105" s="30">
+        <v>1463</v>
       </c>
       <c r="K105" s="22" cm="1">
         <f t="array" ref="K105">F105-G105</f>
@@ -5118,12 +5228,16 @@
         <f t="array" ref="L105">F105-H105</f>
         <v>#VALUE!</v>
       </c>
-      <c r="M105" s="23"/>
+      <c r="M105" s="12">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:M1"/>
   </mergeCells>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup orientation="portrait"/>
   <headerFooter>

</xml_diff>